<commit_message>
Group B: 4005 flange O-rings from the Brennan CAD records (checked on BRENNAN_4005-08), folded into the 4000 ring master: +8 configurations
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sbz7LkX6Jr9QuSxTU76dzT
</commit_message>
<xml_diff>
--- a/tools/_out/groupB_20261021/stage/04_DESIGN_TABLES/DesignTable_4005.xlsx
+++ b/tools/_out/groupB_20261021/stage/04_DESIGN_TABLES/DesignTable_4005.xlsx
@@ -413,43 +413,68 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>OMi 4005 - Design Table SKELETON (no dimensional source) | OMi catalog 9 SKUs | ALL MISSING | GENERATED 2026-09-23</t>
+          <t>OMi 4005 Flange O-Ring (Buna-N) - review table | Brennan CAD records (PARTcommunity, o_rings_and_seals/4005) | group B 2026-10-21 | folded into the 4000 O-ring master</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
+          <t>ID@DRIVE</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>W@DRIVE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>$PRP@DimSource</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>$PRP@Material</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>$PRP@TubeOD</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>$PRP@PartNo</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>$PRP@DataStatus</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>$PRP@AxialSource</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>$PRP@ScopeAction</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>$PRP@OMiSKU</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>$COMMENT</t>
         </is>
@@ -461,34 +486,55 @@
           <t>4005-08</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" t="n">
+        <v>0.734</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Buna-N (Brennan CAD record)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>4005-08</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAD 2026-10-21 group B: ID@DRIVE, W@DRIVE] Brennan CAD record 4005-08 (I.D. 0.734, W 0.14; checked on BRENNAN_4005-08: I.D. 0.734 / O.D. 1.014 / W 0.140); no Air-Way page, no OMi sizes [user 2026-10-21: Brennan CAD records "following my rule"]</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>4005-08</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled</t>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled | Brennan CAD record 4005-08 (PARTcommunity / CADENAS, group B 2026-10-21: ID@DRIVE=ID, W@DRIVE=W; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
     </row>
@@ -498,34 +544,55 @@
           <t>4005-10</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" t="n">
+        <v>0.859</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Buna-N (Brennan CAD record)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>5/8</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>4005-10</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAD 2026-10-21 group B: ID@DRIVE, W@DRIVE] Brennan CAD record 4005-10 (I.D. 0.859, W 0.14; checked on BRENNAN_4005-08: I.D. 0.734 / O.D. 1.014 / W 0.140); no Air-Way page, no OMi sizes [user 2026-10-21: Brennan CAD records "following my rule"]</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>4005-10</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled</t>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled | Brennan CAD record 4005-10 (PARTcommunity / CADENAS, group B 2026-10-21: ID@DRIVE=ID, W@DRIVE=W; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
     </row>
@@ -535,34 +602,55 @@
           <t>4005-12</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" t="n">
+        <v>0.984</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Buna-N (Brennan CAD record)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>4005-12</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAD 2026-10-21 group B: ID@DRIVE, W@DRIVE] Brennan CAD record 4005-12 (I.D. 0.984, W 0.14; checked on BRENNAN_4005-08: I.D. 0.734 / O.D. 1.014 / W 0.140); no Air-Way page, no OMi sizes [user 2026-10-21: Brennan CAD records "following my rule"]</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>4005-12</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled</t>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled | Brennan CAD record 4005-12 (PARTcommunity / CADENAS, group B 2026-10-21: ID@DRIVE=ID, W@DRIVE=W; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
     </row>
@@ -572,34 +660,55 @@
           <t>4005-16</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" t="n">
+        <v>1.296</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Buna-N (Brennan CAD record)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>4005-16</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAD 2026-10-21 group B: ID@DRIVE, W@DRIVE] Brennan CAD record 4005-16 (I.D. 1.296, W 0.14; checked on BRENNAN_4005-08: I.D. 0.734 / O.D. 1.014 / W 0.140); no Air-Way page, no OMi sizes [user 2026-10-21: Brennan CAD records "following my rule"]</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>4005-16</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled</t>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled | Brennan CAD record 4005-16 (PARTcommunity / CADENAS, group B 2026-10-21: ID@DRIVE=ID, W@DRIVE=W; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
     </row>
@@ -609,34 +718,55 @@
           <t>4005-20</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" t="n">
+        <v>1.484</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Buna-N (Brennan CAD record)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1 1/4</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>4005-20</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAD 2026-10-21 group B: ID@DRIVE, W@DRIVE] Brennan CAD record 4005-20 (I.D. 1.484, W 0.14; checked on BRENNAN_4005-08: I.D. 0.734 / O.D. 1.014 / W 0.140); no Air-Way page, no OMi sizes [user 2026-10-21: Brennan CAD records "following my rule"]</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>4005-20</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled</t>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled | Brennan CAD record 4005-20 (PARTcommunity / CADENAS, group B 2026-10-21: ID@DRIVE=ID, W@DRIVE=W; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
     </row>
@@ -646,34 +776,55 @@
           <t>4005-24</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" t="n">
+        <v>1.859</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Buna-N (Brennan CAD record)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1 1/2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>4005-24</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAD 2026-10-21 group B: ID@DRIVE, W@DRIVE] Brennan CAD record 4005-24 (I.D. 1.859, W 0.14; checked on BRENNAN_4005-08: I.D. 0.734 / O.D. 1.014 / W 0.140); no Air-Way page, no OMi sizes [user 2026-10-21: Brennan CAD records "following my rule"]</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>4005-24</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled</t>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled | Brennan CAD record 4005-24 (PARTcommunity / CADENAS, group B 2026-10-21: ID@DRIVE=ID, W@DRIVE=W; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
     </row>
@@ -683,34 +834,55 @@
           <t>4005-32</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" t="n">
+        <v>2.234</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Buna-N (Brennan CAD record)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>4005-32</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAD 2026-10-21 group B: ID@DRIVE, W@DRIVE] Brennan CAD record 4005-32 (I.D. 2.234, W 0.14; checked on BRENNAN_4005-08: I.D. 0.734 / O.D. 1.014 / W 0.140); no Air-Way page, no OMi sizes [user 2026-10-21: Brennan CAD records "following my rule"]</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>4005-32</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled</t>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled | Brennan CAD record 4005-32 (PARTcommunity / CADENAS, group B 2026-10-21: ID@DRIVE=ID, W@DRIVE=W; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
     </row>
@@ -720,34 +892,55 @@
           <t>4005-40</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" t="n">
+        <v>2.734</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Buna-N (Brennan CAD record)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2 1/2</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>4005-40</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>[BRENNAN-CAD 2026-10-21 group B: ID@DRIVE, W@DRIVE] Brennan CAD record 4005-40 (I.D. 2.734, W 0.14; checked on BRENNAN_4005-08: I.D. 0.734 / O.D. 1.014 / W 0.140); no Air-Way page, no OMi sizes [user 2026-10-21: Brennan CAD records "following my rule"]</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>4005-40</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled</t>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled | Brennan CAD record 4005-40 (PARTcommunity / CADENAS, group B 2026-10-21: ID@DRIVE=ID, W@DRIVE=W; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
     </row>
@@ -757,34 +950,34 @@
           <t>4005-48</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>4005-48</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way lists no carbon-steel series for this root -&gt; no dimensions</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>BUILD</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>4005-48</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled</t>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>MISSING: needs a dimensional source (Air-Way sibling family, Parker/Brennan catalog, or a STEP measurement) before any geometry is modelled | group B 2026-10-21: no Brennan CAD record for this size (PARTcommunity returned none) - stays MISSING</t>
         </is>
       </c>
     </row>

</xml_diff>